<commit_message>
rerun model qwen3:8b RAG GOT Model results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_8b/comparison_GoTRAG/GoTRAG_consolidated.xlsx
+++ b/results/qwen3_8b/comparison_GoTRAG/GoTRAG_consolidated.xlsx
@@ -569,7 +569,7 @@
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>0.2586206896551724</v>
@@ -703,7 +703,7 @@
         <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L4" t="n">
         <v>0.3181818181818182</v>
@@ -770,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>0.3037974683544304</v>
@@ -971,7 +971,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>0.2123893805309734</v>
@@ -1038,7 +1038,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L9" t="n">
         <v>0.3134328358208955</v>
@@ -1105,7 +1105,7 @@
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L10" t="n">
         <v>0.3278688524590164</v>
@@ -1172,7 +1172,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>0.2659574468085106</v>
@@ -1306,7 +1306,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
         <v>0.3389830508474576</v>
@@ -1373,7 +1373,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L14" t="n">
         <v>0.3220338983050847</v>
@@ -1507,7 +1507,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L16" t="n">
         <v>0.3163265306122449</v>
@@ -1708,7 +1708,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
         <v>0.2195121951219512</v>
@@ -1775,7 +1775,7 @@
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L20" t="n">
         <v>0.3076923076923077</v>
@@ -1976,7 +1976,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
         <v>0.2666666666666667</v>
@@ -2043,7 +2043,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="L24" t="n">
         <v>0.256</v>
@@ -2110,7 +2110,7 @@
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L25" t="n">
         <v>0.3177570093457944</v>
@@ -2244,7 +2244,7 @@
         <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
         <v>0.2891566265060241</v>
@@ -2378,7 +2378,7 @@
         <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>0.2978723404255319</v>
@@ -2445,7 +2445,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L30" t="n">
         <v>0.264367816091954</v>
@@ -2579,7 +2579,7 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>0.3125</v>
@@ -2646,7 +2646,7 @@
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>0.3</v>
@@ -2713,7 +2713,7 @@
         <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L34" t="n">
         <v>0.2941176470588235</v>
@@ -2780,7 +2780,7 @@
         <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L35" t="n">
         <v>0.2844036697247707</v>
@@ -2847,7 +2847,7 @@
         <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
         <v>0.3962264150943396</v>
@@ -3048,7 +3048,7 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>0.373134328358209</v>
@@ -3249,7 +3249,7 @@
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L42" t="n">
         <v>0.2727272727272727</v>
@@ -3316,7 +3316,7 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="L43" t="n">
         <v>0.3023255813953488</v>
@@ -3450,7 +3450,7 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>0.2708333333333333</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>0.3387096774193548</v>
@@ -3651,7 +3651,7 @@
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
         <v>0.3214285714285715</v>
@@ -3718,7 +3718,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L49" t="n">
         <v>0.264367816091954</v>
@@ -3852,7 +3852,7 @@
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
         <v>0.3392857142857143</v>
@@ -3919,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
         <v>0.2567567567567567</v>
@@ -3986,7 +3986,7 @@
         <v>1</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L53" t="n">
         <v>0.3050847457627119</v>
@@ -4120,7 +4120,7 @@
         <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" t="n">
         <v>0.2571428571428571</v>
@@ -4321,7 +4321,7 @@
         <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="L58" t="n">
         <v>0.3780487804878049</v>
@@ -4388,7 +4388,7 @@
         <v>1</v>
       </c>
       <c r="K59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L59" t="n">
         <v>0.2702702702702703</v>
@@ -4522,7 +4522,7 @@
         <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
         <v>0.2950819672131147</v>
@@ -4589,7 +4589,7 @@
         <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
         <v>0.2982456140350877</v>
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
         <v>0.25</v>
@@ -4723,7 +4723,7 @@
         <v>1</v>
       </c>
       <c r="K64" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="L64" t="n">
         <v>0.2935779816513762</v>
@@ -4857,7 +4857,7 @@
         <v>1</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>0.2746478873239437</v>
@@ -4991,7 +4991,7 @@
         <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>0.2335329341317365</v>

</xml_diff>